<commit_message>
Q07: seed, import fixture and decisions in Portuguese; screenshots regenerated with a pt-BR date input
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNa4LfCZTxuKquPfqR5uPB
</commit_message>
<xml_diff>
--- a/test/fixtures/2026-10-import.xlsx
+++ b/test/fixtures/2026-10-import.xlsx
@@ -461,17 +461,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Marcio salary</t>
+          <t>Salário Marcio</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Salary</t>
+          <t>Salário</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Marcio checking</t>
+          <t>Conta Marcio</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Freelance design</t>
+          <t>Freela de design</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Marcio checking</t>
+          <t>Conta Marcio</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rent</t>
+          <t>Aluguel</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Housing</t>
+          <t>Moradia</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Joint checking</t>
+          <t>Conta conjunta</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -566,17 +566,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Phone plan</t>
+          <t>Plano de celular</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Contas da casa</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Marcio card</t>
+          <t>Cartão Marcio</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -601,17 +601,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Groceries</t>
+          <t>Supermercado</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Groceries</t>
+          <t>Alimentação</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Marcio card</t>
+          <t>Cartão Marcio</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">

</xml_diff>